<commit_message>
Regenerate ASD risk matrices after September 2026 refresh
804 active events, all classified: 90-day refresh merged into restored curated dedup state, Insight marketing page rejected, MediSecure fragment merged.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/risk_matrix/risk_matrix.xlsx
+++ b/risk_matrix/risk_matrix.xlsx
@@ -27,11 +27,11 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -68,10 +68,10 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -509,7 +509,7 @@
         <v>21</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="G2" s="4" t="n">
         <v>1</v>
@@ -528,13 +528,13 @@
         <v>2</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>207</v>
+        <v>223</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>72</v>
+        <v>83</v>
       </c>
       <c r="G3" s="4" t="n">
         <v>3</v>
@@ -547,19 +547,19 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>189</v>
+        <v>222</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="G4" s="3" t="inlineStr"/>
     </row>
@@ -588,16 +588,16 @@
         <v>3</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E6" s="4" t="n">
         <v>24</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G6" s="3" t="inlineStr"/>
     </row>
@@ -611,19 +611,19 @@
         <v>33</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="D7" s="4" t="n">
         <v>28</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>107</v>
+        <v>124</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Regenerate ASD risk matrices after October 2026 refresh
832 active events, all classified: 90-day refresh merged incrementally into curated dedup state (24 into existing, 29 new); Way Forward fragment merged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/risk_matrix/risk_matrix.xlsx
+++ b/risk_matrix/risk_matrix.xlsx
@@ -531,10 +531,10 @@
         <v>22</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="G3" s="4" t="n">
         <v>3</v>
@@ -550,16 +550,16 @@
         <v>10</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G4" s="3" t="inlineStr"/>
     </row>
@@ -588,16 +588,16 @@
         <v>3</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D6" s="4" t="n">
         <v>23</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G6" s="3" t="inlineStr"/>
     </row>
@@ -608,19 +608,19 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="G7" s="4" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
Regenerate ASD risk matrices after Sharp Motor Group clean-up
Sharp Motor Group held 13 foreign records (9 unrelated Cyber Daily articles, 4 Sharp Office Systems); they were split out via dedup_admin split and folded into their own incidents, Sharp Motor re-dated to 2026-08-23 by member consensus.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/risk_matrix/risk_matrix.xlsx
+++ b/risk_matrix/risk_matrix.xlsx
@@ -531,7 +531,7 @@
         <v>22</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F3" s="4" t="n">
         <v>85</v>
@@ -553,7 +553,7 @@
         <v>25</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E4" s="4" t="n">
         <v>227</v>
@@ -591,7 +591,7 @@
         <v>22</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E6" s="4" t="n">
         <v>26</v>

</xml_diff>

<commit_message>
Recurrence analyses and risk matrices from snapshot snap-20261030171144
Refresh of 2026-10-30: 621 pages discovered, duplicate check re-run cleanly (16 more
merges), evidence recovery (12 incidents unsupported, from 169). 182 repeats; adjusted
constant-hazard p = 0.152 with ties collapsed, 0.040 with the 5 remaining ties as repeats.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/risk_matrix/risk_matrix.xlsx
+++ b/risk_matrix/risk_matrix.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risk Matrix" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Not placed" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -66,7 +67,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -79,6 +80,9 @@
     </xf>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -502,18 +506,14 @@
       </c>
       <c r="B2" s="3" t="inlineStr"/>
       <c r="C2" s="3" t="inlineStr"/>
-      <c r="D2" s="4" t="n">
+      <c r="D2" s="3" t="inlineStr"/>
+      <c r="E2" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E2" s="4" t="n">
-        <v>23</v>
-      </c>
       <c r="F2" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="G2" s="4" t="n">
-        <v>1</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="G2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -522,22 +522,20 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="C3" s="4" t="n">
-        <v>2</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="C3" s="3" t="inlineStr"/>
       <c r="D3" s="4" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>233</v>
+        <v>118</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>85</v>
+        <v>18</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -547,21 +545,23 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>104</v>
+        <v>167</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>230</v>
+        <v>202</v>
       </c>
       <c r="F4" s="4" t="n">
         <v>49</v>
       </c>
-      <c r="G4" s="3" t="inlineStr"/>
+      <c r="G4" s="4" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -569,14 +569,24 @@
           <t>Coordinated low-level malicious attack</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr"/>
-      <c r="C5" s="3" t="inlineStr"/>
-      <c r="D5" s="3" t="inlineStr"/>
+      <c r="B5" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="E5" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F5" s="3" t="inlineStr"/>
-      <c r="G5" s="3" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -585,19 +595,19 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C6" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>24</v>
-      </c>
       <c r="E6" s="4" t="n">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="G6" s="3" t="inlineStr"/>
     </row>
@@ -608,22 +618,289 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>34</v>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>29</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr"/>
       <c r="E7" s="4" t="n">
-        <v>135</v>
+        <v>4</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="G7" s="4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Impact Type</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Stakeholder</t>
+        </is>
+      </c>
+      <c r="C1" s="5" t="inlineStr">
+        <is>
+          <t>Classifications</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Coordinated low-level malicious attack</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Insufficient information</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Extensive compromise</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Insufficient information</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Insufficient information</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Academia/R&amp;D</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Insufficient information</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Federal government</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Insufficient information</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Insufficient information</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Insufficient information</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Large organisation(s)</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Insufficient information</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Member(s) of the public</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Insufficient information</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>National security</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Insufficient information</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Regulated critical infrastructure</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Insufficient information</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Schools</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Insufficient information</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Small organisation(s)</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Insufficient information</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>State government</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Insufficient information</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Supply chain</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
         <v>10</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Isolated compromise</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Insufficient information</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Low-level malicious attack</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Insufficient information</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Unsuccessful low-level malicious attack</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Insufficient information</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Recurrence analyses on snapshot snap-20261030202652 (labels applied, scope recalibrated)
Labelled non-incidents rejected and labelled-real events restored through merges; event scope at its new
0.68 cut-off. 165 repeats; adjusted constant-hazard p = 0.174 with ties collapsed, 0.063 with the 4
remaining ties as separate repeats. Quality gate passed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/risk_matrix/risk_matrix.xlsx
+++ b/risk_matrix/risk_matrix.xlsx
@@ -529,7 +529,7 @@
         <v>24</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F3" s="4" t="n">
         <v>18</v>
@@ -554,7 +554,7 @@
         <v>167</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="F4" s="4" t="n">
         <v>49</v>
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>4</v>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7">
@@ -750,7 +750,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8">
@@ -765,7 +765,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">

</xml_diff>

<commit_message>
Analyses and risk matrices on snapshot snap-20261031122958 (supplier per-customer split, descriptions unfolded, labelled victims filled)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/risk_matrix/risk_matrix.xlsx
+++ b/risk_matrix/risk_matrix.xlsx
@@ -508,10 +508,10 @@
       <c r="C2" s="3" t="inlineStr"/>
       <c r="D2" s="3" t="inlineStr"/>
       <c r="E2" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G2" s="3" t="inlineStr"/>
     </row>
@@ -522,17 +522,17 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
       <c r="D3" s="4" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="G3" s="4" t="n">
         <v>4</v>
@@ -545,19 +545,19 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>167</v>
+        <v>178</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G4" s="4" t="n">
         <v>2</v>
@@ -570,7 +570,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>1</v>
@@ -578,11 +578,9 @@
       <c r="D5" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="4" t="n">
-        <v>2</v>
-      </c>
+      <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5" s="4" t="n">
         <v>2</v>
@@ -604,7 +602,7 @@
         <v>3</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F6" s="4" t="n">
         <v>8</v>
@@ -643,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -690,7 +688,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4">
@@ -735,7 +733,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7">
@@ -750,7 +748,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8">
@@ -761,11 +759,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Member(s) of the public</t>
+          <t>Local government</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -776,11 +774,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>National security</t>
+          <t>Medium-sized organisation(s)</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -791,11 +789,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Regulated critical infrastructure</t>
+          <t>Member(s) of the public</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -806,11 +804,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Schools</t>
+          <t>National security</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12">
@@ -821,11 +819,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Small organisation(s)</t>
+          <t>Regulated critical infrastructure</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
@@ -836,11 +834,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>State government</t>
+          <t>Schools</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -851,47 +849,47 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Supply chain</t>
+          <t>Small organisation(s)</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Isolated compromise</t>
+          <t>Insufficient information</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Insufficient information</t>
+          <t>State government</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>79</v>
+        <v>5</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Low-level malicious attack</t>
+          <t>Insufficient information</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Insufficient information</t>
+          <t>Supply chain</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Unsuccessful low-level malicious attack</t>
+          <t>Isolated compromise</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -900,7 +898,22 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1</v>
+        <v>74</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Low-level malicious attack</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Insufficient information</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Analyses and risk matrices on snapshot snap-20261031184502 (supplier registry repaired, Finance pair merged)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/risk_matrix/risk_matrix.xlsx
+++ b/risk_matrix/risk_matrix.xlsx
@@ -522,14 +522,14 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C3" s="3" t="inlineStr"/>
       <c r="D3" s="4" t="n">
         <v>22</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="F3" s="4" t="n">
         <v>16</v>
@@ -554,10 +554,10 @@
         <v>178</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G4" s="4" t="n">
         <v>2</v>

</xml_diff>